<commit_message>
write_off page | 06092026
</commit_message>
<xml_diff>
--- a/TSD_smart.xlsx
+++ b/TSD_smart.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,688 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5473547457</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0104905601008805215ybpTstOh*hJb</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-09-03 13:50:42</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0104027816299349215MF!r2?M3rv5C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:27:40</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0104027816299349215CcWhfXxlwrEP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:27:40</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PCF2001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0104027816299349215g5pSieoztY5/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-09-05 10:44:52</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>jj</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0104650532210741215oUIWsUEC6qfw</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:32:26</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PCF2001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0104027816299349215%HGYTluTaeT=</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-09-05 11:52:29</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PCF2001</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0104027816299349215&lt;pum+Lq=wcpb</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-09-05 11:52:29</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G004000M2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0104027816390701215&lt;Sm!UFs=W:&amp;a</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:29:18</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0104008177182372215"PN_ME-u;uuQ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0104008177182372215"daa:CoUIUoz</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0104008177182372215%VSHSe1mqklH</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0104008177182372215&amp;ZnkW,!MmwFD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0104008177182372215&amp;cKAP?8Jls0&lt;</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0104008177182372215&amp;d?jG/FNZljt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0104008177182372215'zNGp5&amp;C2abu</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0104008177182372215(kqsOTNIgFP?</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0104008177182372215)PCDmCehG&gt;Qd</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0104008177182372215*QTb_YuDkiVD</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0104008177182372215*p9Egp8XirOV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0104008177182372215+OdQ8UpK2rUc</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0104008177182372215,4cDiw+kf9i3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0104008177182372215,P?fMIAWqYFC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0104008177182372215,sNXUr*E&amp;h9?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0104008177182372215.BcXj)Jj&lt;/aE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>G3504</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0104008177182372215.Q.IJlskzopu</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:12</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0104008177182372215.doU5JcIgKXp</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:40:52</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PG51183</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0104008177182372215/qiU0"q=auLU</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:34:40</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0104008177182372215/h&lt;E")Yfmaoc</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-09-05 12:40:52</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>01040081771823722152xi6M&amp;5P'WBr</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:27:40</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>01040081771823722155n9ateK7XNdr</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:27:40</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GS65577F2EUR</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>010400817718237221571MJtnS7vSip</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:27:40</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>